<commit_message>
chore: actualizar dossier y dashboard 2026-10-11
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,32 +567,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -647,18 +647,18 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
@@ -745,11 +745,11 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -843,11 +843,11 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -941,11 +941,11 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1039,11 +1039,11 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1137,11 +1137,11 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1155,7 +1155,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1230,30 +1230,30 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1333,18 +1333,18 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S9" t="n">
         <v>79</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1435,21 +1435,21 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1529,25 +1529,25 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="S11" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1627,18 +1627,18 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
         <v>31</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S13" t="n">
         <v>76</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S23" t="n">
         <v>76</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>66</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S25" t="n">
         <v>65</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>63</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S29" t="n">
         <v>63</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3801,32 +3801,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3866,65 +3866,67 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-10</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S35" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3964,65 +3966,67 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-10</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="n">
-        <v>7305</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S36" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4077,7 +4081,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4090,39 +4094,39 @@
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4177,7 +4181,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4186,18 +4190,18 @@
         </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4207,7 +4211,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4222,7 +4226,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4277,7 +4281,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4286,43 +4290,43 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4381,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,18 +4390,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4411,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4417,12 +4421,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4432,12 +4436,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4477,7 +4481,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,18 +4490,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4507,7 +4511,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4522,7 +4526,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4532,12 +4536,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4586,18 +4590,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4611,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4621,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4636,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4686,18 +4690,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4711,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4721,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4736,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,18 +4790,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4817,12 +4821,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4836,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4886,18 +4890,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4907,7 +4911,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4917,12 +4921,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Quid 16. Revista del Área de Estudios Urbanos</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4932,12 +4936,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4957,7 +4961,7 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -4986,18 +4990,18 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Quid 16</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5007,7 +5011,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5017,12 +5021,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Quid 16. Revista del Área de Estudios Urbanos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5057,7 +5061,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5086,109 +5090,9 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5242,7 +5146,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-12
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -665,7 +665,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -675,22 +675,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -749,46 +749,46 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S3" t="n">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -847,14 +847,14 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
@@ -945,14 +945,14 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -1043,14 +1043,14 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -1141,46 +1141,46 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1230,30 +1230,30 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1333,18 +1333,18 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="S9" t="n">
         <v>79</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
@@ -1435,21 +1435,21 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1524,30 +1524,30 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="S11" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1627,25 +1627,25 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>177</v>
+        <v>81</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>207</v>
+        <v>176</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>308</v>
+        <v>215</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>359</v>
+        <v>312</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3866,67 +3866,65 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-10-05</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>358</v>
       </c>
       <c r="S35" t="n">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3966,67 +3964,65 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-12</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>7305</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4066,67 +4062,65 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-12</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>7305</v>
       </c>
       <c r="S37" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4181,7 +4175,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4190,18 +4184,18 @@
         </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4211,7 +4205,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4221,12 +4215,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4281,7 +4275,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4290,18 +4284,18 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4311,7 +4305,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4321,12 +4315,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4381,7 +4375,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4394,39 +4388,39 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4436,12 +4430,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4481,7 +4475,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4490,18 +4484,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4521,12 +4515,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4536,12 +4530,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4581,7 +4575,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4590,18 +4584,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4611,7 +4605,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4621,7 +4615,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4690,18 +4684,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4711,7 +4705,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4721,12 +4715,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4794,14 +4788,14 @@
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4811,7 +4805,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4821,12 +4815,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4836,12 +4830,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4890,18 +4884,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Quid 16</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4911,7 +4905,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4921,12 +4915,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Quid 16. Revista del Área de Estudios Urbanos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4936,12 +4930,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4961,7 +4955,7 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -4990,109 +4984,409 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Delito y Sociedad</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>78</v>
+      </c>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Quid 16</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>sociología, política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Quid 16. Revista del Área de Estudios Urbanos</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>70</v>
+      </c>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="T47" s="4" t="inlineStr">
+      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5146,6 +5440,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-13
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S3" t="n">
         <v>74</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>64</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S9" t="n">
         <v>79</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>79</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>52</v>
@@ -1645,7 +1645,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="S13" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="S21" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S23" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S25" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S27" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>81</v>
+        <v>175</v>
       </c>
       <c r="S29" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>215</v>
+        <v>306</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2046-10-13</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>358</v>
+        <v>7305</v>
       </c>
       <c r="S35" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-12</t>
+          <t>2046-10-13</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3990,39 +3990,39 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,65 +4062,67 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-12</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S37" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4175,7 +4177,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4188,14 +4190,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4205,7 +4207,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4215,12 +4217,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4288,39 +4290,39 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4375,7 +4377,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4384,43 +4386,43 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4475,7 +4477,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4484,18 +4486,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4505,7 +4507,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4515,12 +4517,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4575,7 +4577,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4584,18 +4586,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4605,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4615,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4630,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4684,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4705,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4715,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4730,12 +4732,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4784,18 +4786,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4805,7 +4807,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4815,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4888,14 +4890,14 @@
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4905,7 +4907,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4915,12 +4917,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4984,18 +4986,18 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5015,7 +5017,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5084,309 +5086,9 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Quid 16</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Quid 16. Revista del Área de Estudios Urbanos</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>70</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5440,9 +5142,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-14
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
         <v>74</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>64</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1253,7 +1253,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1333,25 +1333,25 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="S9" t="n">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1431,18 +1431,18 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
@@ -1533,21 +1533,21 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1622,30 +1622,30 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1725,25 +1725,25 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1823,18 +1823,18 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2607,50 +2607,50 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,46 +2709,46 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>175</v>
+        <v>79</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>205</v>
+        <v>79</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>214</v>
+        <v>174</v>
       </c>
       <c r="S31" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>306</v>
+        <v>204</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>311</v>
+        <v>213</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>357</v>
+        <v>305</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3836,12 +3836,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3881,50 +3881,50 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-13</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>7305</v>
+        <v>310</v>
       </c>
       <c r="S35" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3979,50 +3979,50 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-13</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>7305</v>
+        <v>356</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,67 +4062,65 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-14</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>7305</v>
       </c>
       <c r="S37" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4162,67 +4160,65 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-14</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>7305</v>
       </c>
       <c r="S38" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4277,7 +4273,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4290,39 +4286,39 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4373,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,18 +4382,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4403,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4422,7 +4418,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4477,7 +4473,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,43 +4482,43 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4577,7 +4573,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4586,18 +4582,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4603,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4613,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4628,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4677,7 +4673,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4686,18 +4682,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4703,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,7 +4713,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4786,18 +4782,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4807,7 +4803,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4817,12 +4813,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4890,14 +4886,14 @@
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4907,7 +4903,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4917,12 +4913,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4932,12 +4928,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4986,109 +4982,409 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Contextos de Educación</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Río Cuarto</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>educación, política</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>68</v>
+      </c>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Delito y Sociedad</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>64</v>
+      </c>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="T47" s="4" t="inlineStr">
+      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5142,6 +5438,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-15
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3" t="n">
         <v>74</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>64</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,10 +1435,10 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S13" t="n">
         <v>52</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>79</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S21" t="n">
         <v>76</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>76</v>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S23" t="n">
         <v>68</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>68</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S25" t="n">
         <v>76</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>66</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S27" t="n">
         <v>65</v>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>63</v>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S29" t="n">
         <v>55</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>55</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S31" t="n">
         <v>63</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>76</v>
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="R35" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="S35" t="n">
         <v>76</v>
@@ -3983,7 +3983,7 @@
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="S36" s="2" t="n">
         <v>49</v>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-14</t>
+          <t>2046-10-15</t>
         </is>
       </c>
       <c r="R37" t="n">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2046-10-14</t>
+          <t>2046-10-15</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-16
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,32 +567,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -647,25 +647,25 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -675,22 +675,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -749,46 +749,46 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S3" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -847,14 +847,14 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -945,14 +945,14 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -1043,14 +1043,14 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
@@ -1141,46 +1141,46 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1230,23 +1230,23 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R9" t="n">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
@@ -1645,7 +1645,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1725,25 +1725,25 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="S13" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1823,18 +1823,18 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="S21" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2607,50 +2607,50 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,46 +2709,46 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S23" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S25" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S27" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>78</v>
+        <v>172</v>
       </c>
       <c r="S29" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>78</v>
+        <v>202</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>173</v>
+        <v>211</v>
       </c>
       <c r="S31" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>203</v>
+        <v>303</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>212</v>
+        <v>308</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>304</v>
+        <v>354</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3836,12 +3836,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3881,50 +3881,50 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2046-10-16</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>309</v>
+        <v>7305</v>
       </c>
       <c r="S35" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3979,50 +3979,50 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2046-10-16</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>355</v>
+        <v>7305</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,65 +4062,67 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-15</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S37" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4160,65 +4162,67 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2046-10-15</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>7305</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4273,7 +4277,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4286,39 +4290,39 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4373,7 +4377,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4382,18 +4386,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4403,7 +4407,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4418,7 +4422,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4473,7 +4477,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4482,43 +4486,43 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4573,7 +4577,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4582,18 +4586,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4603,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4613,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4628,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4673,7 +4677,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4682,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4703,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4713,7 +4717,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4782,18 +4786,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4803,7 +4807,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4813,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4886,14 +4890,14 @@
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4903,7 +4907,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4913,12 +4917,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4928,12 +4932,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4982,18 +4986,18 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5003,7 +5007,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5013,12 +5017,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5028,12 +5032,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5082,309 +5086,9 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Delito y Sociedad</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>64</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5438,9 +5142,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-17
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
@@ -1645,7 +1645,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>172</v>
+        <v>76</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>202</v>
+        <v>171</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>303</v>
+        <v>210</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>354</v>
+        <v>307</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-16</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>7305</v>
+        <v>353</v>
       </c>
       <c r="S35" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-16</t>
+          <t>2046-10-17</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3990,39 +3990,39 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,67 +4062,65 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-17</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>7305</v>
       </c>
       <c r="S37" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4177,7 +4175,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4190,14 +4188,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4207,7 +4205,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4217,12 +4215,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4290,39 +4288,39 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4375,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,43 +4384,43 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4477,7 +4475,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,11 +4484,11 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4695,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4705,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4715,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4730,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,18 +4784,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4807,7 +4805,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4817,12 +4815,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4830,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4886,18 +4884,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4917,12 +4915,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4932,12 +4930,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4986,109 +4984,209 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>64</v>
+      </c>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O48" s="2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="T47" s="4" t="inlineStr">
+      <c r="T48" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5142,6 +5240,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-18
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -647,11 +647,11 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -745,11 +745,11 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -843,11 +843,11 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -941,11 +941,11 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1039,11 +1039,11 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1137,11 +1137,11 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,10 +1533,10 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S11" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
@@ -1631,10 +1631,10 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="S13" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="S21" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
+        <v>75</v>
+      </c>
+      <c r="S23" t="n">
         <v>76</v>
       </c>
-      <c r="S23" t="n">
-        <v>68</v>
-      </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S25" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S27" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>76</v>
+        <v>170</v>
       </c>
       <c r="S29" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>210</v>
+        <v>301</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>307</v>
+        <v>352</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2046-10-18</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>353</v>
+        <v>7305</v>
       </c>
       <c r="S35" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-17</t>
+          <t>2046-10-18</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3990,39 +3990,39 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,65 +4062,67 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-17</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S37" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4175,7 +4177,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4188,14 +4190,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4205,7 +4207,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4215,12 +4217,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4288,39 +4290,39 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4375,7 +4377,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4384,43 +4386,43 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4475,7 +4477,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4484,11 +4486,11 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4597,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4605,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4615,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4630,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4684,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4705,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4715,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4788,14 +4790,14 @@
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4805,7 +4807,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4815,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4884,18 +4886,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4915,7 +4917,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4984,209 +4986,9 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
-        <v>64</v>
-      </c>
-      <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5239,8 +5041,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-19
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S11" t="n">
         <v>82</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>82</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S13" t="n">
         <v>76</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S23" t="n">
         <v>76</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>66</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S25" t="n">
         <v>65</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>63</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S29" t="n">
         <v>63</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-18</t>
+          <t>2046-10-19</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-18</t>
+          <t>2046-10-19</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -4597,7 +4597,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4686,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,18 +4786,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4817,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4832,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4886,109 +4886,209 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O46" s="2" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P46" s="2" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n">
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
         <v>57</v>
       </c>
-      <c r="T46" s="3" t="inlineStr">
+      <c r="T47" s="4" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5041,6 +5141,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-20
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="S11" t="n">
         <v>82</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>82</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S13" t="n">
         <v>76</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S23" t="n">
         <v>76</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>66</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S25" t="n">
         <v>65</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>63</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S29" t="n">
         <v>63</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-19</t>
+          <t>2046-10-20</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-19</t>
+          <t>2046-10-20</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-21
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -665,32 +665,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -749,14 +749,14 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -847,14 +847,14 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -945,14 +945,14 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
@@ -1043,46 +1043,46 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1141,14 +1141,14 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S7" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1246,14 +1246,14 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1328,30 +1328,30 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S9" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1431,18 +1431,18 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
@@ -1533,21 +1533,21 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="S11" t="n">
         <v>82</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1622,23 +1622,23 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1729,14 +1729,14 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S13" t="n">
         <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,46 +2317,46 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2411,50 +2411,50 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,46 +2513,46 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2611,21 +2611,21 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,25 +3195,25 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>73</v>
+        <v>167</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>207</v>
+        <v>298</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,50 +3685,50 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>304</v>
+        <v>349</v>
       </c>
       <c r="S33" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3783,18 +3783,18 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2046-10-21</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>350</v>
+        <v>7305</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-20</t>
+          <t>2046-10-21</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3892,39 +3892,39 @@
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3964,65 +3964,67 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-20</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S36" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4077,7 +4079,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4090,14 +4092,14 @@
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -4107,7 +4109,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -4117,12 +4119,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4190,39 +4192,39 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4277,7 +4279,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4286,43 +4288,43 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4379,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,18 +4388,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4409,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4417,12 +4419,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4477,7 +4479,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,18 +4488,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4507,7 +4509,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4517,12 +4519,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4532,12 +4534,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4586,18 +4588,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4609,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4619,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4634,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4686,18 +4688,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4709,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4719,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4734,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,18 +4788,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4817,12 +4819,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4834,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4886,18 +4888,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4917,12 +4919,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4932,12 +4934,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4986,109 +4988,9 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
-        <v>57</v>
-      </c>
-      <c r="T47" s="4" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5141,7 +5043,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-22
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3" t="n">
         <v>66</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" t="n">
         <v>55</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1253,7 +1253,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1333,18 +1333,18 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S9" t="n">
         <v>82</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
@@ -1435,46 +1435,46 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1524,55 +1524,55 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="S11" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1627,25 +1627,25 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,25 +1725,25 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1823,25 +1823,25 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1921,25 +1921,25 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="S15" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2019,25 +2019,25 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>51</v>
+        <v>166</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2117,25 +2117,25 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>51</v>
+        <v>205</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2155,12 +2155,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2215,25 +2215,25 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>51</v>
+        <v>297</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2313,40 +2313,40 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>51</v>
+        <v>348</v>
       </c>
       <c r="S19" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2411,50 +2411,50 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2046-10-22</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>72</v>
+        <v>7305</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2046-10-22</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>72</v>
+        <v>7305</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2592,40 +2592,42 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R22" s="2" t="n">
-        <v>72</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S22" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2637,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,12 +2647,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2662,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2690,40 +2692,42 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R23" t="n">
-        <v>72</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S23" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2737,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,12 +2747,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2762,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2788,40 +2792,42 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R24" s="2" t="n">
-        <v>72</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S24" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2837,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2847,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2856,12 +2862,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2886,40 +2892,42 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R25" t="n">
-        <v>72</v>
+          <t>5000-10-01</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S25" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2937,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,12 +2947,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2954,12 +2962,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2984,40 +2992,42 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R26" s="2" t="n">
-        <v>72</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S26" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3037,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,12 +3047,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3082,40 +3092,42 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="R27" t="n">
-        <v>72</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3137,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3147,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3150,12 +3162,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3180,40 +3192,42 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
-        </is>
-      </c>
-      <c r="R28" s="2" t="n">
-        <v>167</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S28" s="2" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3237,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3247,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3278,40 +3292,42 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
-        </is>
-      </c>
-      <c r="R29" t="n">
-        <v>197</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S29" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3337,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3347,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3346,12 +3362,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3376,40 +3392,42 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
-        </is>
-      </c>
-      <c r="R30" s="2" t="n">
-        <v>206</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S30" s="2" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3437,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3447,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3474,1523 +3492,33 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
-        </is>
-      </c>
-      <c r="R31" t="n">
-        <v>298</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S31" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Revista Análisis de las Prácticas</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>educación, sociología, política, humanidades</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="Q32" s="2" t="inlineStr">
-        <is>
-          <t>2027-08-20</t>
-        </is>
-      </c>
-      <c r="R32" s="2" t="n">
-        <v>303</v>
-      </c>
-      <c r="S32" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="T32" s="3" t="inlineStr">
-        <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Mendoza</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>educación, política, humanidades</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>2027-10-05</t>
-        </is>
-      </c>
-      <c r="R33" t="n">
-        <v>349</v>
-      </c>
-      <c r="S33" t="n">
-        <v>49</v>
-      </c>
-      <c r="T33" s="4" t="inlineStr">
-        <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Políticas Educativas – PolEd</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Porto Alegre</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Mercosur</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>educación, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Políticas Educativas – PolEd</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t>2046-10-21</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="n">
-        <v>7305</v>
-      </c>
-      <c r="S34" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="T34" s="3" t="inlineStr">
-        <is>
-          <t>https://seer.ufrgs.br/poled</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Políticas Educativas – PolEd</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Porto Alegre</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Mercosur</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>educación, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Políticas Educativas – PolEd</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>abierta</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>2046-10-21</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>7305</v>
-      </c>
-      <c r="S35" t="n">
-        <v>68</v>
-      </c>
-      <c r="T35" s="4" t="inlineStr">
-        <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Historia y Sociedad</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Medellín</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Historia y sociedad</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S36" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="T36" s="3" t="inlineStr">
-        <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Del prudente Saber</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Paraná</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S37" t="n">
-        <v>70</v>
-      </c>
-      <c r="T37" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Cuadernos del CIESAL</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Rosario</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S38" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="T38" s="3" t="inlineStr">
-        <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Revista Exitus</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Santarém</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>educación, política</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Anúncios</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>2027-02-15</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S39" t="n">
-        <v>55</v>
-      </c>
-      <c r="T39" s="4" t="inlineStr">
-        <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Envíos</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q40" s="2" t="inlineStr">
-        <is>
-          <t>5000-10-01</t>
-        </is>
-      </c>
-      <c r="R40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S40" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="T40" s="3" t="inlineStr">
-        <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Raigal</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Villa María</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S41" t="n">
-        <v>70</v>
-      </c>
-      <c r="T41" s="4" t="inlineStr">
-        <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Revista de educación (Mar del Plata)</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Mar del Plata</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>educación, sociología, humanidades</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S42" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T42" s="3" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Contextos de Educación</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Río Cuarto</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>educación, política</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S43" t="n">
-        <v>68</v>
-      </c>
-      <c r="T43" s="4" t="inlineStr">
-        <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Delito y Sociedad</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S44" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T44" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S45" t="n">
-        <v>64</v>
-      </c>
-      <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T46" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5028,21 +3556,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-23
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -665,32 +665,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -749,14 +749,14 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S3" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
@@ -847,14 +847,14 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -945,14 +945,14 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -1043,46 +1043,46 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1141,14 +1141,14 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1235,25 +1235,25 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1328,30 +1328,30 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="S9" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1426,55 +1426,55 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1524,55 +1524,55 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="S11" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1622,30 +1622,30 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,25 +1725,25 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="S13" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1823,25 +1823,25 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1921,25 +1921,25 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="S15" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2019,25 +2019,25 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>166</v>
+        <v>49</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2117,25 +2117,25 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>205</v>
+        <v>49</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2155,12 +2155,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2215,25 +2215,25 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>297</v>
+        <v>49</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2313,50 +2313,50 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>348</v>
+        <v>49</v>
       </c>
       <c r="S19" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2411,40 +2411,40 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2046-10-22</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>7305</v>
+        <v>49</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2509,25 +2509,25 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2046-10-22</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>7305</v>
+        <v>70</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2592,42 +2592,40 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="n">
+        <v>70</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2637,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2647,12 +2645,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2662,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2692,42 +2690,40 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R23" t="n">
+        <v>70</v>
       </c>
       <c r="S23" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2737,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2747,12 +2743,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2762,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2792,42 +2788,40 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>70</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2837,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2847,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2862,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2892,42 +2886,40 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R25" t="n">
+        <v>70</v>
       </c>
       <c r="S25" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2937,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2947,12 +2939,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2962,12 +2954,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2992,42 +2984,40 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>70</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3037,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3047,12 +3037,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3092,42 +3082,40 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>70</v>
       </c>
       <c r="S27" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3137,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3147,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3162,12 +3150,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3192,42 +3180,40 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>70</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3237,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3247,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3292,42 +3278,40 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-04-06</t>
+        </is>
+      </c>
+      <c r="R29" t="n">
+        <v>165</v>
       </c>
       <c r="S29" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3337,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3347,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3362,12 +3346,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3392,133 +3376,1619 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-05-06</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>195</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>De Prácticas y Discursos</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Corrientes</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>2027-05-15</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>204</v>
+      </c>
+      <c r="S31" t="n">
+        <v>76</v>
+      </c>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Revista SAAP</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Revista Análisis de las Prácticas</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>educación, sociología, política, humanidades</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>2027-08-20</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>301</v>
+      </c>
+      <c r="S33" t="n">
+        <v>76</v>
+      </c>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Traslaciones / convocatoria UNCuyo</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>educación, política, humanidades</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>2027-10-05</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>347</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Políticas Educativas – PolEd</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Mercosur</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>educación, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Políticas Educativas – PolEd</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>2046-10-23</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>7305</v>
+      </c>
+      <c r="S35" t="n">
+        <v>68</v>
+      </c>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>https://seer.ufrgs.br/poled</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Políticas Educativas – PolEd</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Mercosur</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>educación, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Políticas Educativas – PolEd</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>2046-10-23</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>7305</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Historia y Sociedad</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>sociología, política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Historia y sociedad</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S37" t="n">
+        <v>70</v>
+      </c>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Del prudente Saber</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Paraná</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Cuadernos del CIESAL</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S39" t="n">
+        <v>70</v>
+      </c>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Envíos</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>5000-10-01</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Raigal</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Villa María</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S41" t="n">
+        <v>70</v>
+      </c>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Revista de educación (Mar del Plata)</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Mar del Plata</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>educación, sociología, humanidades</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="T42" s="3" t="inlineStr">
+        <is>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Contextos de Educación</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Río Cuarto</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>educación, política</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S43" t="n">
+        <v>68</v>
+      </c>
+      <c r="T43" s="4" t="inlineStr">
+        <is>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Delito y Sociedad</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="T44" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S45" t="n">
+        <v>64</v>
+      </c>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O46" s="2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S31" t="n">
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="T31" s="4" t="inlineStr">
+      <c r="T46" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -3556,6 +5026,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-24
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>66</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>66</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>55</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" t="n">
         <v>55</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>82</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S11" t="n">
         <v>82</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>82</v>
@@ -1645,7 +1645,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,14 +3199,14 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S29" t="n">
         <v>63</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-23</t>
+          <t>2046-10-24</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-23</t>
+          <t>2046-10-24</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -4597,7 +4597,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4686,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,211 +4786,11 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S45" t="n">
-        <v>64</v>
-      </c>
-      <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T46" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -5039,8 +4839,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-25
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,32 +567,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -647,50 +647,50 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -745,50 +745,50 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -843,50 +843,50 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -896,12 +896,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -941,50 +941,50 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S5" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1039,50 +1039,50 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1137,50 +1137,50 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S7" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1235,50 +1235,50 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1333,50 +1333,50 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S9" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1431,50 +1431,50 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1533,21 +1533,21 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S11" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1627,25 +1627,25 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1725,18 +1725,18 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="S13" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,14 +2317,14 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2509,50 +2509,50 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="S21" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S23" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S25" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S27" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,14 +3199,14 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="S29" t="n">
         <v>63</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3801,32 +3801,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-24</t>
+          <t>2027-10-25</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>7305</v>
+        <v>365</v>
       </c>
       <c r="S35" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-24</t>
+          <t>2046-10-25</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3990,39 +3990,39 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,67 +4062,65 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2046-10-25</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>7305</v>
       </c>
       <c r="S37" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4177,7 +4175,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4190,14 +4188,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4207,7 +4205,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4217,12 +4215,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4290,14 +4288,14 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4307,7 +4305,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4322,7 +4320,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4375,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,18 +4384,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4405,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4417,12 +4415,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4477,7 +4475,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,18 +4484,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4507,7 +4505,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4517,12 +4515,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4532,12 +4530,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4586,18 +4584,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4605,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4615,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4690,7 +4688,7 @@
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
@@ -4791,6 +4789,306 @@
       <c r="T44" s="3" t="inlineStr">
         <is>
           <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Delito y Sociedad</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S45" t="n">
+        <v>78</v>
+      </c>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>57</v>
+      </c>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
       </c>
     </row>
@@ -4839,6 +5137,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-26
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -647,25 +647,25 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -685,12 +685,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -745,18 +745,18 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
@@ -847,46 +847,46 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>82</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -896,12 +896,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -945,21 +945,21 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -969,22 +969,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1043,46 +1043,46 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1141,14 +1141,14 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S7" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -1239,14 +1239,14 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -1337,14 +1337,14 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
@@ -1435,46 +1435,46 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1524,30 +1524,30 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="S11" t="n">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1622,23 +1622,23 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1729,14 +1729,14 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S13" t="n">
         <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S15" t="n">
         <v>76</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S17" t="n">
         <v>76</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,46 +2317,46 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2411,50 +2411,50 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,46 +2513,46 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2611,21 +2611,21 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,25 +3195,25 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>68</v>
+        <v>162</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>202</v>
+        <v>293</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,18 +3685,18 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>299</v>
+        <v>344</v>
       </c>
       <c r="S33" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3783,18 +3783,18 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-10-25</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-10-25</t>
+          <t>2027-10-26</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-25</t>
+          <t>2046-10-26</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-25</t>
+          <t>2046-10-26</t>
         </is>
       </c>
       <c r="R37" t="n">

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-27
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>82</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S5" t="n">
         <v>74</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>64</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>66</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1547,7 +1547,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1622,23 +1622,23 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1729,14 +1729,14 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S13" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S15" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S17" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,46 +2317,46 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S19" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2411,50 +2411,50 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,46 +2513,46 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2611,21 +2611,21 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S23" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S25" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,25 +3195,25 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>162</v>
+        <v>66</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>192</v>
+        <v>161</v>
       </c>
       <c r="S29" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>293</v>
+        <v>200</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,18 +3685,18 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>344</v>
+        <v>297</v>
       </c>
       <c r="S33" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3783,18 +3783,18 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-25</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-10-26</t>
+          <t>2027-10-25</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="S35" t="n">
         <v>49</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-26</t>
+          <t>2046-10-27</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-26</t>
+          <t>2046-10-27</t>
         </is>
       </c>
       <c r="R37" t="n">

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-28
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>82</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
         <v>74</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>64</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>66</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1547,7 +1547,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1622,23 +1622,23 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1729,14 +1729,14 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S13" t="n">
         <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S15" t="n">
         <v>79</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S17" t="n">
         <v>79</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2219,14 +2219,14 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2317,46 +2317,46 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S19" t="n">
         <v>79</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2411,50 +2411,50 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,46 +2513,46 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2611,21 +2611,21 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
+        <v>65</v>
+      </c>
+      <c r="S23" t="n">
         <v>66</v>
       </c>
-      <c r="S23" t="n">
-        <v>76</v>
-      </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S25" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,25 +3195,25 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>66</v>
+        <v>160</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>200</v>
+        <v>291</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,18 +3685,18 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>297</v>
+        <v>342</v>
       </c>
       <c r="S33" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-10-25</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-10-25</t>
+          <t>2046-10-28</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>363</v>
+        <v>7305</v>
       </c>
       <c r="S35" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-27</t>
+          <t>2046-10-28</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3990,39 +3990,39 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,65 +4062,67 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2046-10-27</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>7305</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S37" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4175,7 +4177,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4188,14 +4190,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4205,7 +4207,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4215,12 +4217,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4288,14 +4290,14 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4305,7 +4307,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4320,7 +4322,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4375,7 +4377,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4384,18 +4386,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4405,7 +4407,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4415,12 +4417,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4475,7 +4477,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4484,18 +4486,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4505,7 +4507,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4515,12 +4517,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4530,12 +4532,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4584,18 +4586,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4605,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4615,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4630,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4684,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4705,7 +4707,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4715,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4730,12 +4732,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4784,18 +4786,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4815,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4830,12 +4832,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4884,18 +4886,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4915,12 +4917,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4930,12 +4932,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4984,109 +4986,9 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
-        <v>57</v>
-      </c>
-      <c r="T47" s="4" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5139,7 +5041,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-29
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>82</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S5" t="n">
         <v>74</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>64</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>66</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S13" t="n">
         <v>79</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>79</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S15" t="n">
         <v>79</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>79</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S17" t="n">
         <v>79</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>79</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S19" t="n">
         <v>79</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>68</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>76</v>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S23" t="n">
         <v>66</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>65</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S25" t="n">
         <v>63</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>55</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S27" t="n">
         <v>55</v>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>63</v>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="S29" t="n">
         <v>76</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>76</v>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="S31" t="n">
         <v>76</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="S33" t="n">
         <v>49</v>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>49</v>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-28</t>
+          <t>2046-10-29</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-28</t>
+          <t>2046-10-29</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -4297,7 +4297,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4317,12 +4317,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,18 +4386,18 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4417,12 +4417,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4432,12 +4432,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4486,18 +4486,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4517,12 +4517,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4532,12 +4532,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4586,18 +4586,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4617,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4632,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4686,18 +4686,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4786,18 +4786,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4817,12 +4817,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4832,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4886,109 +4886,9 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T46" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5040,7 +4940,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-30
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -647,18 +647,18 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
@@ -749,46 +749,46 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -847,21 +847,21 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -871,22 +871,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -945,46 +945,46 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1043,14 +1043,14 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
@@ -1141,14 +1141,14 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
@@ -1239,14 +1239,14 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
@@ -1337,46 +1337,46 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1426,23 +1426,23 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S13" t="n">
         <v>79</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>79</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S15" t="n">
         <v>79</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>79</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S17" t="n">
         <v>79</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>79</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S19" t="n">
         <v>79</v>
@@ -2331,22 +2331,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2415,46 +2415,46 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,46 +2513,46 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>TEMÁTICO nº 01/2027- La reforma de la educación secundaria: desafíos y contradicciones</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2709,46 +2709,46 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S23" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2258</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2807,46 +2807,46 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S25" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,25 +3195,25 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>159</v>
+        <v>63</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3293,25 +3293,25 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>189</v>
+        <v>63</v>
       </c>
       <c r="S29" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>198</v>
+        <v>63</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>290</v>
+        <v>63</v>
       </c>
       <c r="S31" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>295</v>
+        <v>158</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>341</v>
+        <v>188</v>
       </c>
       <c r="S33" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,50 +3783,50 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-10-25</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>361</v>
+        <v>197</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3836,12 +3836,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3881,50 +3881,50 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2046-10-29</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>7305</v>
+        <v>289</v>
       </c>
       <c r="S35" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3979,50 +3979,50 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2046-10-29</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>7305</v>
+        <v>294</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4062,42 +4062,40 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-10-05</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>340</v>
       </c>
       <c r="S37" t="n">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -4107,7 +4105,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -4117,12 +4115,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4162,67 +4160,65 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>permanente</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>continua</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2027-10-25</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>360</v>
       </c>
       <c r="S38" s="2" t="n">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4277,7 +4273,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4290,14 +4286,14 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4307,7 +4303,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4317,12 +4313,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4373,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4390,14 +4386,14 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4407,7 +4403,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4417,12 +4413,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4432,12 +4428,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4477,7 +4473,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4486,33 +4482,33 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4522,7 +4518,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4577,7 +4573,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4586,18 +4582,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4607,7 +4603,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4617,12 +4613,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4628,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4677,7 +4673,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4686,18 +4682,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4707,7 +4703,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4717,12 +4713,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4786,109 +4782,609 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>Revista de educación (Mar del Plata)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Mar del Plata</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>educación, sociología, humanidades</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S45" t="n">
+        <v>78</v>
+      </c>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Historia de la Educación. Anuario</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Anuario de Historia de la Educación</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Contextos de Educación</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Río Cuarto</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>educación, política</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>68</v>
+      </c>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Delito y Sociedad</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>sociología, política, ciencias sociales</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Sobre la revista</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>NBRA</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>CAICYT-CONICET</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>El Taco en la Brea</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>política, humanidades</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Para autores</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>permanente</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>continua</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>64</v>
+      </c>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Sobre la revista</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>NBRA</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>CAICYT-CONICET</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>permanente</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>continua</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S45" t="n">
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="T45" s="4" t="inlineStr">
+      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -4940,6 +5436,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-10-31
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>82</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>82</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>74</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>64</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>66</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>66</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>66</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
         <v>66</v>
@@ -1351,7 +1351,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1431,25 +1431,25 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Prórroga del Dossier "Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1524,23 +1524,23 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="S11" t="n">
         <v>79</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1631,14 +1631,14 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
@@ -1729,14 +1729,14 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S13" t="n">
         <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S15" t="n">
         <v>79</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S17" t="n">
         <v>79</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2219,46 +2219,46 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>79</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2313,18 +2313,18 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="S19" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
@@ -2415,14 +2415,14 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2513,14 +2513,14 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S21" t="n">
         <v>68</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
         </is>
       </c>
     </row>
@@ -2547,12 +2547,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>TEMÁTICO nº 01/2027- La reforma de la educación secundaria: desafíos y contradicciones</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2258</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>TEMÁTICO nº 01/2027- La reforma de la educación secundaria: desafíos y contradicciones</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2709,46 +2709,46 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S23" t="n">
         <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2258</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2807,46 +2807,46 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S25" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S27" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="S28" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="S28" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3297,21 +3297,21 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S29" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -3395,21 +3395,21 @@
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>55</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3429,12 +3429,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R31" t="n">
+        <v>157</v>
+      </c>
+      <c r="S31" t="n">
         <v>63</v>
       </c>
-      <c r="S31" t="n">
-        <v>55</v>
-      </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="S33" t="n">
         <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3783,25 +3783,25 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>197</v>
+        <v>288</v>
       </c>
       <c r="S34" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3821,12 +3821,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,25 +3881,25 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="S35" t="n">
         <v>76</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3979,18 +3979,18 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
+          <t>2027-10-05</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>294</v>
+        <v>339</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4077,50 +4077,50 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2027-10-05</t>
+          <t>2027-10-25</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="S37" t="n">
         <v>49</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora de Empresas UNCuyo abre una nueva  para transformar ideas en empresas</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4160,65 +4160,67 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2027-10-25</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>360</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/la-incubadora-de-empresas-uncuyo-abre-una-nueva-convocatoria-para-transformar-ideas-en-empresas</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4273,7 +4275,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4286,14 +4288,14 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4303,7 +4305,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4313,12 +4315,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4386,39 +4388,39 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4473,7 +4475,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4482,43 +4484,43 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4573,7 +4575,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>5000-10-01</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4582,18 +4584,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4603,7 +4605,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4613,12 +4615,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4673,7 +4675,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>5000-10-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4682,18 +4684,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4703,7 +4705,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4713,12 +4715,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4728,12 +4730,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4782,18 +4784,18 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4803,7 +4805,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4813,12 +4815,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4828,12 +4830,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4882,18 +4884,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4903,7 +4905,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4913,12 +4915,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Anuario de Historia de la Educación</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4986,14 +4988,14 @@
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5003,7 +5005,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5013,12 +5015,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5082,18 +5084,18 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/user/setLocale/en?source=%2Fojs%2Findex.php%2Fcontextos%2Fannouncement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -5113,7 +5115,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -5182,209 +5184,9 @@
         </is>
       </c>
       <c r="S48" s="2" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>64</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5439,8 +5241,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>